<commit_message>
Fix cell formatting in templates
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/BOEStatusWithUCOTByBOE.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/BOEStatusWithUCOTByBOE.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A812CB63-4592-4F2F-99E4-409AD2C5E9CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D0735F-ADAD-407A-8AFE-05E91EE0A91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1785" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE Status - BOEs Only" sheetId="1" r:id="rId1"/>
@@ -136,7 +136,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -148,6 +148,12 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -464,9 +470,9 @@
     <col min="5" max="5" width="25.7109375" style="1" customWidth="1"/>
     <col min="6" max="7" width="15.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="13.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23.5703125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="25.7109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="20.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="23.5703125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="25.7109375" style="4" customWidth="1"/>
+    <col min="11" max="11" width="20.28515625" style="6" customWidth="1"/>
     <col min="12" max="12" width="22.5703125" style="1" customWidth="1"/>
     <col min="13" max="13" width="20.42578125" style="1" customWidth="1"/>
     <col min="14" max="14" width="17.85546875" style="1" customWidth="1"/>
@@ -506,7 +512,7 @@
       <c r="J1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="2" t="s">

</xml_diff>